<commit_message>
added Operator ID section
added operator ID section and tidied up numbering system and table of contents
</commit_message>
<xml_diff>
--- a/Images for Markdown files database updated 30-06-2026.xlsx
+++ b/Images for Markdown files database updated 30-06-2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trevor\Compac Industries\Compac - General\IT\ChatBot\Markdown-Manuals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD687A7-09BE-4A9E-BB08-7D832916EFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC362D2-0ADC-4A02-B3EF-31690F3305B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-1320" windowWidth="38640" windowHeight="21120" xr2:uid="{7323B22B-375C-41F7-91CD-F86C900FC6DE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="711">
   <si>
     <t xml:space="preserve">PCBs </t>
   </si>
@@ -2147,6 +2147,36 @@
   </si>
   <si>
     <t>Mechanical  - Pumps</t>
+  </si>
+  <si>
+    <t>Gateway</t>
+  </si>
+  <si>
+    <t>20.1.1</t>
+  </si>
+  <si>
+    <t>20.1.2</t>
+  </si>
+  <si>
+    <t>20.1.1_GW_image.png</t>
+  </si>
+  <si>
+    <t>20.1.2_GW_LITE_image.png</t>
+  </si>
+  <si>
+    <t>front page image</t>
+  </si>
+  <si>
+    <t>20.1.3</t>
+  </si>
+  <si>
+    <t>20.1.3_GW_arch_image.png</t>
+  </si>
+  <si>
+    <t>architecture image</t>
+  </si>
+  <si>
+    <t>Comfill Ex (Volume Register) specific</t>
   </si>
 </sst>
 </file>
@@ -2184,7 +2214,7 @@
       <name val="HelveticaNeue LT 57 Cn"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2236,6 +2266,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2293,7 +2329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2387,6 +2423,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2721,14 +2764,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B533B56-556A-40A2-8D3F-E8E5A852019A}">
-  <dimension ref="A1:K347"/>
+  <dimension ref="A1:K373"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.7265625" customWidth="1"/>
     <col min="3" max="3" width="10.6328125" style="1" customWidth="1"/>
     <col min="4" max="4" width="47.26953125" customWidth="1"/>
-    <col min="5" max="5" width="11.6328125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.7265625" customWidth="1"/>
     <col min="7" max="11" width="11.6328125" customWidth="1"/>
   </cols>
@@ -5635,6 +5678,9 @@
       <c r="G179" s="5"/>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B181" t="s">
+        <v>696</v>
+      </c>
       <c r="C181" s="1" t="s">
         <v>594</v>
       </c>
@@ -6043,143 +6089,46 @@
         <v>676</v>
       </c>
     </row>
-    <row r="262" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A262" s="20"/>
-      <c r="B262" s="21"/>
-      <c r="C262" s="20"/>
-      <c r="D262" s="21"/>
-      <c r="E262" s="20"/>
-      <c r="F262" s="21"/>
-      <c r="G262" s="21"/>
-      <c r="H262" s="21"/>
-      <c r="I262" s="21"/>
-      <c r="J262" s="21"/>
-      <c r="K262" s="21"/>
-    </row>
     <row r="263" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A263" s="22">
+      <c r="B263" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="268" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A268" s="20"/>
+      <c r="B268" s="21"/>
+      <c r="C268" s="20"/>
+      <c r="D268" s="21"/>
+      <c r="E268" s="20"/>
+      <c r="F268" s="21"/>
+      <c r="G268" s="21"/>
+      <c r="H268" s="21"/>
+      <c r="I268" s="21"/>
+      <c r="J268" s="21"/>
+      <c r="K268" s="21"/>
+    </row>
+    <row r="269" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A269" s="22">
         <v>13</v>
       </c>
-      <c r="B263" s="23" t="s">
+      <c r="B269" s="23" t="s">
         <v>677</v>
       </c>
-      <c r="C263" s="22" t="s">
+      <c r="C269" s="22" t="s">
         <v>678</v>
       </c>
-      <c r="D263" s="24" t="s">
+      <c r="D269" s="24" t="s">
         <v>684</v>
       </c>
-      <c r="E263" s="22" t="s">
+      <c r="E269" s="22" t="s">
         <v>696</v>
       </c>
-      <c r="F263" s="22" t="s">
+      <c r="F269" s="22" t="s">
         <v>697</v>
       </c>
-      <c r="G263" s="24" t="s">
+      <c r="G269" s="24" t="s">
         <v>698</v>
       </c>
-      <c r="H263" s="24"/>
-      <c r="I263" s="24"/>
-      <c r="J263" s="24"/>
-      <c r="K263" s="24"/>
-    </row>
-    <row r="264" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A264" s="22"/>
-      <c r="B264" s="24"/>
-      <c r="C264" s="22" t="s">
-        <v>679</v>
-      </c>
-      <c r="D264" s="24" t="s">
-        <v>686</v>
-      </c>
-      <c r="E264" s="22"/>
-      <c r="F264" s="24"/>
-      <c r="G264" s="24"/>
-      <c r="H264" s="24"/>
-      <c r="I264" s="24"/>
-      <c r="J264" s="24"/>
-      <c r="K264" s="24"/>
-    </row>
-    <row r="265" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A265" s="22"/>
-      <c r="B265" s="24"/>
-      <c r="C265" s="22" t="s">
-        <v>680</v>
-      </c>
-      <c r="D265" s="24" t="s">
-        <v>685</v>
-      </c>
-      <c r="E265" s="22"/>
-      <c r="F265" s="24"/>
-      <c r="G265" s="24"/>
-      <c r="H265" s="24"/>
-      <c r="I265" s="24"/>
-      <c r="J265" s="24"/>
-      <c r="K265" s="24"/>
-    </row>
-    <row r="266" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A266" s="22"/>
-      <c r="B266" s="24"/>
-      <c r="C266" s="22" t="s">
-        <v>681</v>
-      </c>
-      <c r="D266" s="24" t="s">
-        <v>687</v>
-      </c>
-      <c r="E266" s="22"/>
-      <c r="F266" s="24"/>
-      <c r="G266" s="24"/>
-      <c r="H266" s="24"/>
-      <c r="I266" s="24"/>
-      <c r="J266" s="24"/>
-      <c r="K266" s="24"/>
-    </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A267" s="22"/>
-      <c r="B267" s="24"/>
-      <c r="C267" s="22" t="s">
-        <v>682</v>
-      </c>
-      <c r="D267" s="24" t="s">
-        <v>688</v>
-      </c>
-      <c r="E267" s="22"/>
-      <c r="F267" s="24"/>
-      <c r="G267" s="24"/>
-      <c r="H267" s="24"/>
-      <c r="I267" s="24"/>
-      <c r="J267" s="24"/>
-      <c r="K267" s="24"/>
-    </row>
-    <row r="268" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A268" s="22"/>
-      <c r="B268" s="24"/>
-      <c r="C268" s="22" t="s">
-        <v>683</v>
-      </c>
-      <c r="D268" s="24" t="s">
-        <v>689</v>
-      </c>
-      <c r="E268" s="22"/>
-      <c r="F268" s="24"/>
-      <c r="G268" s="24"/>
-      <c r="H268" s="24"/>
-      <c r="I268" s="24"/>
-      <c r="J268" s="24"/>
-      <c r="K268" s="24"/>
-    </row>
-    <row r="269" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A269" s="22"/>
-      <c r="B269" s="24"/>
-      <c r="C269" s="22" t="s">
-        <v>690</v>
-      </c>
-      <c r="D269" s="24" t="s">
-        <v>693</v>
-      </c>
-      <c r="E269" s="22"/>
-      <c r="F269" s="24"/>
-      <c r="G269" s="24"/>
       <c r="H269" s="24"/>
       <c r="I269" s="24"/>
       <c r="J269" s="24"/>
@@ -6189,10 +6138,10 @@
       <c r="A270" s="22"/>
       <c r="B270" s="24"/>
       <c r="C270" s="22" t="s">
-        <v>691</v>
+        <v>679</v>
       </c>
       <c r="D270" s="24" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="E270" s="22"/>
       <c r="F270" s="24"/>
@@ -6206,10 +6155,10 @@
       <c r="A271" s="22"/>
       <c r="B271" s="24"/>
       <c r="C271" s="22" t="s">
-        <v>692</v>
+        <v>680</v>
       </c>
       <c r="D271" s="24" t="s">
-        <v>695</v>
+        <v>685</v>
       </c>
       <c r="E271" s="22"/>
       <c r="F271" s="24"/>
@@ -6222,8 +6171,12 @@
     <row r="272" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A272" s="22"/>
       <c r="B272" s="24"/>
-      <c r="C272" s="22"/>
-      <c r="D272" s="24"/>
+      <c r="C272" s="22" t="s">
+        <v>681</v>
+      </c>
+      <c r="D272" s="24" t="s">
+        <v>687</v>
+      </c>
       <c r="E272" s="22"/>
       <c r="F272" s="24"/>
       <c r="G272" s="24"/>
@@ -6233,306 +6186,302 @@
       <c r="K272" s="24"/>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A273" s="20"/>
-      <c r="B273" s="21"/>
-      <c r="C273" s="20"/>
-      <c r="D273" s="21"/>
-      <c r="E273" s="20"/>
-      <c r="F273" s="21"/>
-      <c r="G273" s="21"/>
-      <c r="H273" s="21"/>
-      <c r="I273" s="21"/>
-      <c r="J273" s="21"/>
-      <c r="K273" s="21"/>
-    </row>
-    <row r="282" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C282" s="1" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C283" s="1" t="s">
-        <v>520</v>
-      </c>
-      <c r="D283" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="284" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C284" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="D284" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="285" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C285" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="D285" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="286" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C286" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="D286" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="287" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C287" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="D287" t="s">
-        <v>525</v>
-      </c>
+      <c r="A273" s="22"/>
+      <c r="B273" s="24"/>
+      <c r="C273" s="22" t="s">
+        <v>682</v>
+      </c>
+      <c r="D273" s="24" t="s">
+        <v>688</v>
+      </c>
+      <c r="E273" s="22"/>
+      <c r="F273" s="24"/>
+      <c r="G273" s="24"/>
+      <c r="H273" s="24"/>
+      <c r="I273" s="24"/>
+      <c r="J273" s="24"/>
+      <c r="K273" s="24"/>
+    </row>
+    <row r="274" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A274" s="22"/>
+      <c r="B274" s="24"/>
+      <c r="C274" s="22" t="s">
+        <v>683</v>
+      </c>
+      <c r="D274" s="24" t="s">
+        <v>689</v>
+      </c>
+      <c r="E274" s="22"/>
+      <c r="F274" s="24"/>
+      <c r="G274" s="24"/>
+      <c r="H274" s="24"/>
+      <c r="I274" s="24"/>
+      <c r="J274" s="24"/>
+      <c r="K274" s="24"/>
+    </row>
+    <row r="275" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A275" s="22"/>
+      <c r="B275" s="24"/>
+      <c r="C275" s="22" t="s">
+        <v>690</v>
+      </c>
+      <c r="D275" s="24" t="s">
+        <v>693</v>
+      </c>
+      <c r="E275" s="22"/>
+      <c r="F275" s="24"/>
+      <c r="G275" s="24"/>
+      <c r="H275" s="24"/>
+      <c r="I275" s="24"/>
+      <c r="J275" s="24"/>
+      <c r="K275" s="24"/>
+    </row>
+    <row r="276" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A276" s="22"/>
+      <c r="B276" s="24"/>
+      <c r="C276" s="22" t="s">
+        <v>691</v>
+      </c>
+      <c r="D276" s="24" t="s">
+        <v>694</v>
+      </c>
+      <c r="E276" s="22"/>
+      <c r="F276" s="24"/>
+      <c r="G276" s="24"/>
+      <c r="H276" s="24"/>
+      <c r="I276" s="24"/>
+      <c r="J276" s="24"/>
+      <c r="K276" s="24"/>
+    </row>
+    <row r="277" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A277" s="22"/>
+      <c r="B277" s="24"/>
+      <c r="C277" s="22" t="s">
+        <v>692</v>
+      </c>
+      <c r="D277" s="24" t="s">
+        <v>695</v>
+      </c>
+      <c r="E277" s="22"/>
+      <c r="F277" s="24"/>
+      <c r="G277" s="24"/>
+      <c r="H277" s="24"/>
+      <c r="I277" s="24"/>
+      <c r="J277" s="24"/>
+      <c r="K277" s="24"/>
+    </row>
+    <row r="278" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A278" s="22"/>
+      <c r="B278" s="24"/>
+      <c r="C278" s="22"/>
+      <c r="D278" s="24"/>
+      <c r="E278" s="22"/>
+      <c r="F278" s="24"/>
+      <c r="G278" s="24"/>
+      <c r="H278" s="24"/>
+      <c r="I278" s="24"/>
+      <c r="J278" s="24"/>
+      <c r="K278" s="24"/>
+    </row>
+    <row r="279" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A279" s="20"/>
+      <c r="B279" s="21"/>
+      <c r="C279" s="20"/>
+      <c r="D279" s="21"/>
+      <c r="E279" s="20"/>
+      <c r="F279" s="21"/>
+      <c r="G279" s="21"/>
+      <c r="H279" s="21"/>
+      <c r="I279" s="21"/>
+      <c r="J279" s="21"/>
+      <c r="K279" s="21"/>
     </row>
     <row r="288" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C288" s="1" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="289" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C289" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="D289" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="290" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C290" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="D290" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="291" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C291" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="D291" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="292" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C292" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="D292" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="293" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C293" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="D293" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="294" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C294" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="D288" t="s">
+      <c r="D294" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="289" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C289" s="1" t="s">
+    <row r="295" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C295" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="D289" t="s">
+      <c r="D295" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="290" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C290" s="1" t="s">
+    <row r="296" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C296" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="D290" t="s">
+      <c r="D296" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="291" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C291" s="1" t="s">
+    <row r="297" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C297" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="D291" t="s">
+      <c r="D297" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="292" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C292" s="1" t="s">
+    <row r="298" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C298" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="D292" t="s">
+      <c r="D298" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="293" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C293" s="1" t="s">
+    <row r="299" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C299" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="D293" t="s">
+      <c r="D299" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="294" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C294" s="1" t="s">
+    <row r="300" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C300" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="D294" t="s">
+      <c r="D300" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="295" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C295" s="1" t="s">
+    <row r="301" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C301" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="D295" t="s">
+      <c r="D301" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="296" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C296" s="1" t="s">
+    <row r="302" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C302" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="D296" t="s">
+      <c r="D302" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="297" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C297" s="1" t="s">
+    <row r="303" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C303" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="D297" t="s">
+      <c r="D303" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="298" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C298" s="1" t="s">
+    <row r="304" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C304" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="D298" t="s">
+      <c r="D304" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="299" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C299" s="1" t="s">
+    <row r="305" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C305" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="D299" t="s">
+      <c r="D305" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="300" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C300" s="1" t="s">
+    <row r="306" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C306" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="D300" t="s">
+      <c r="D306" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="301" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="D301" t="s">
+    <row r="307" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="D307" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="302" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A302" s="26"/>
-      <c r="B302" s="25"/>
-      <c r="C302" s="26"/>
-      <c r="D302" s="25"/>
-      <c r="E302" s="26"/>
-      <c r="F302" s="25"/>
-      <c r="G302" s="25"/>
-      <c r="H302" s="25"/>
-      <c r="I302" s="25"/>
-      <c r="J302" s="25"/>
-      <c r="K302" s="25"/>
-    </row>
-    <row r="303" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A303" s="39">
+    <row r="308" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A308" s="26"/>
+      <c r="B308" s="25"/>
+      <c r="C308" s="26"/>
+      <c r="D308" s="25"/>
+      <c r="E308" s="26"/>
+      <c r="F308" s="25"/>
+      <c r="G308" s="25"/>
+      <c r="H308" s="25"/>
+      <c r="I308" s="25"/>
+      <c r="J308" s="25"/>
+      <c r="K308" s="25"/>
+    </row>
+    <row r="309" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A309" s="39">
         <v>16</v>
       </c>
-      <c r="B303" s="40" t="s">
+      <c r="B309" s="40" t="s">
         <v>516</v>
       </c>
-      <c r="C303" s="41" t="s">
+      <c r="C309" s="41" t="s">
         <v>468</v>
       </c>
-      <c r="D303" s="42" t="s">
+      <c r="D309" s="42" t="s">
         <v>480</v>
       </c>
-      <c r="E303" s="39" t="s">
+      <c r="E309" s="39" t="s">
         <v>696</v>
       </c>
-      <c r="F303" s="42" t="s">
+      <c r="F309" s="42" t="s">
         <v>516</v>
       </c>
-      <c r="G303" s="42"/>
-      <c r="H303" s="42"/>
-      <c r="I303" s="42"/>
-      <c r="J303" s="42"/>
-      <c r="K303" s="42"/>
-    </row>
-    <row r="304" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A304" s="39"/>
-      <c r="B304" s="42"/>
-      <c r="C304" s="41" t="s">
-        <v>469</v>
-      </c>
-      <c r="D304" s="42" t="s">
-        <v>481</v>
-      </c>
-      <c r="E304" s="39"/>
-      <c r="F304" s="42"/>
-      <c r="G304" s="42"/>
-      <c r="H304" s="42"/>
-      <c r="I304" s="42"/>
-      <c r="J304" s="42"/>
-      <c r="K304" s="42"/>
-    </row>
-    <row r="305" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A305" s="39"/>
-      <c r="B305" s="42"/>
-      <c r="C305" s="41" t="s">
-        <v>470</v>
-      </c>
-      <c r="D305" s="42" t="s">
-        <v>482</v>
-      </c>
-      <c r="E305" s="39"/>
-      <c r="F305" s="42"/>
-      <c r="G305" s="42"/>
-      <c r="H305" s="42"/>
-      <c r="I305" s="42"/>
-      <c r="J305" s="42"/>
-      <c r="K305" s="42"/>
-    </row>
-    <row r="306" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A306" s="39"/>
-      <c r="B306" s="42"/>
-      <c r="C306" s="41" t="s">
-        <v>471</v>
-      </c>
-      <c r="D306" s="42" t="s">
-        <v>483</v>
-      </c>
-      <c r="E306" s="39"/>
-      <c r="F306" s="42"/>
-      <c r="G306" s="42"/>
-      <c r="H306" s="42"/>
-      <c r="I306" s="42"/>
-      <c r="J306" s="42"/>
-      <c r="K306" s="42"/>
-    </row>
-    <row r="307" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A307" s="39"/>
-      <c r="B307" s="42"/>
-      <c r="C307" s="41" t="s">
-        <v>472</v>
-      </c>
-      <c r="D307" s="42" t="s">
-        <v>484</v>
-      </c>
-      <c r="E307" s="39"/>
-      <c r="F307" s="42"/>
-      <c r="G307" s="42"/>
-      <c r="H307" s="42"/>
-      <c r="I307" s="42"/>
-      <c r="J307" s="42"/>
-      <c r="K307" s="42"/>
-    </row>
-    <row r="308" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A308" s="39"/>
-      <c r="B308" s="42"/>
-      <c r="C308" s="41" t="s">
-        <v>473</v>
-      </c>
-      <c r="D308" s="42" t="s">
-        <v>485</v>
-      </c>
-      <c r="E308" s="39"/>
-      <c r="F308" s="42"/>
-      <c r="G308" s="42"/>
-      <c r="H308" s="42"/>
-      <c r="I308" s="42"/>
-      <c r="J308" s="42"/>
-      <c r="K308" s="42"/>
-    </row>
-    <row r="309" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A309" s="39"/>
-      <c r="B309" s="42"/>
-      <c r="C309" s="41" t="s">
-        <v>474</v>
-      </c>
-      <c r="D309" s="42" t="s">
-        <v>486</v>
-      </c>
-      <c r="E309" s="39"/>
-      <c r="F309" s="42"/>
       <c r="G309" s="42"/>
       <c r="H309" s="42"/>
       <c r="I309" s="42"/>
@@ -6543,10 +6492,10 @@
       <c r="A310" s="39"/>
       <c r="B310" s="42"/>
       <c r="C310" s="41" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="D310" s="42" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="E310" s="39"/>
       <c r="F310" s="42"/>
@@ -6560,10 +6509,10 @@
       <c r="A311" s="39"/>
       <c r="B311" s="42"/>
       <c r="C311" s="41" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="D311" s="42" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="E311" s="39"/>
       <c r="F311" s="42"/>
@@ -6577,10 +6526,10 @@
       <c r="A312" s="39"/>
       <c r="B312" s="42"/>
       <c r="C312" s="41" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="D312" s="42" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="E312" s="39"/>
       <c r="F312" s="42"/>
@@ -6594,10 +6543,10 @@
       <c r="A313" s="39"/>
       <c r="B313" s="42"/>
       <c r="C313" s="41" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="D313" s="42" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="E313" s="39"/>
       <c r="F313" s="42"/>
@@ -6611,10 +6560,10 @@
       <c r="A314" s="39"/>
       <c r="B314" s="42"/>
       <c r="C314" s="41" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="D314" s="42" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="E314" s="39"/>
       <c r="F314" s="42"/>
@@ -6628,10 +6577,10 @@
       <c r="A315" s="39"/>
       <c r="B315" s="42"/>
       <c r="C315" s="41" t="s">
-        <v>503</v>
+        <v>474</v>
       </c>
       <c r="D315" s="42" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="E315" s="39"/>
       <c r="F315" s="42"/>
@@ -6645,10 +6594,10 @@
       <c r="A316" s="39"/>
       <c r="B316" s="42"/>
       <c r="C316" s="41" t="s">
-        <v>504</v>
+        <v>475</v>
       </c>
       <c r="D316" s="42" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="E316" s="39"/>
       <c r="F316" s="42"/>
@@ -6662,10 +6611,10 @@
       <c r="A317" s="39"/>
       <c r="B317" s="42"/>
       <c r="C317" s="41" t="s">
-        <v>505</v>
+        <v>476</v>
       </c>
       <c r="D317" s="42" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="E317" s="39"/>
       <c r="F317" s="42"/>
@@ -6679,10 +6628,10 @@
       <c r="A318" s="39"/>
       <c r="B318" s="42"/>
       <c r="C318" s="41" t="s">
-        <v>506</v>
+        <v>477</v>
       </c>
       <c r="D318" s="42" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="E318" s="39"/>
       <c r="F318" s="42"/>
@@ -6696,10 +6645,10 @@
       <c r="A319" s="39"/>
       <c r="B319" s="42"/>
       <c r="C319" s="41" t="s">
-        <v>507</v>
+        <v>478</v>
       </c>
       <c r="D319" s="42" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="E319" s="39"/>
       <c r="F319" s="42"/>
@@ -6713,10 +6662,10 @@
       <c r="A320" s="39"/>
       <c r="B320" s="42"/>
       <c r="C320" s="41" t="s">
-        <v>508</v>
+        <v>479</v>
       </c>
       <c r="D320" s="42" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="E320" s="39"/>
       <c r="F320" s="42"/>
@@ -6730,10 +6679,10 @@
       <c r="A321" s="39"/>
       <c r="B321" s="42"/>
       <c r="C321" s="41" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="D321" s="42" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="E321" s="39"/>
       <c r="F321" s="42"/>
@@ -6747,10 +6696,10 @@
       <c r="A322" s="39"/>
       <c r="B322" s="42"/>
       <c r="C322" s="41" t="s">
-        <v>510</v>
+        <v>504</v>
       </c>
       <c r="D322" s="42" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="E322" s="39"/>
       <c r="F322" s="42"/>
@@ -6764,10 +6713,10 @@
       <c r="A323" s="39"/>
       <c r="B323" s="42"/>
       <c r="C323" s="41" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="D323" s="42" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="E323" s="39"/>
       <c r="F323" s="42"/>
@@ -6781,10 +6730,10 @@
       <c r="A324" s="39"/>
       <c r="B324" s="42"/>
       <c r="C324" s="41" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="D324" s="42" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="E324" s="39"/>
       <c r="F324" s="42"/>
@@ -6798,10 +6747,10 @@
       <c r="A325" s="39"/>
       <c r="B325" s="42"/>
       <c r="C325" s="41" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="D325" s="42" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="E325" s="39"/>
       <c r="F325" s="42"/>
@@ -6815,10 +6764,10 @@
       <c r="A326" s="39"/>
       <c r="B326" s="42"/>
       <c r="C326" s="41" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="D326" s="42" t="s">
-        <v>515</v>
+        <v>497</v>
       </c>
       <c r="E326" s="39"/>
       <c r="F326" s="42"/>
@@ -6829,192 +6778,210 @@
       <c r="K326" s="42"/>
     </row>
     <row r="327" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A327" s="26"/>
-      <c r="B327" s="25"/>
-      <c r="C327" s="26"/>
-      <c r="D327" s="25"/>
-      <c r="E327" s="26"/>
-      <c r="F327" s="25"/>
-      <c r="G327" s="25"/>
-      <c r="H327" s="25"/>
-      <c r="I327" s="25"/>
-      <c r="J327" s="25"/>
-      <c r="K327" s="25"/>
+      <c r="A327" s="39"/>
+      <c r="B327" s="42"/>
+      <c r="C327" s="41" t="s">
+        <v>509</v>
+      </c>
+      <c r="D327" s="42" t="s">
+        <v>498</v>
+      </c>
+      <c r="E327" s="39"/>
+      <c r="F327" s="42"/>
+      <c r="G327" s="42"/>
+      <c r="H327" s="42"/>
+      <c r="I327" s="42"/>
+      <c r="J327" s="42"/>
+      <c r="K327" s="42"/>
     </row>
     <row r="328" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A328" s="32"/>
-      <c r="B328" s="33" t="s">
+      <c r="A328" s="39"/>
+      <c r="B328" s="42"/>
+      <c r="C328" s="41" t="s">
+        <v>510</v>
+      </c>
+      <c r="D328" s="42" t="s">
+        <v>499</v>
+      </c>
+      <c r="E328" s="39"/>
+      <c r="F328" s="42"/>
+      <c r="G328" s="42"/>
+      <c r="H328" s="42"/>
+      <c r="I328" s="42"/>
+      <c r="J328" s="42"/>
+      <c r="K328" s="42"/>
+    </row>
+    <row r="329" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A329" s="39"/>
+      <c r="B329" s="42"/>
+      <c r="C329" s="41" t="s">
+        <v>511</v>
+      </c>
+      <c r="D329" s="42" t="s">
+        <v>500</v>
+      </c>
+      <c r="E329" s="39"/>
+      <c r="F329" s="42"/>
+      <c r="G329" s="42"/>
+      <c r="H329" s="42"/>
+      <c r="I329" s="42"/>
+      <c r="J329" s="42"/>
+      <c r="K329" s="42"/>
+    </row>
+    <row r="330" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A330" s="39"/>
+      <c r="B330" s="42"/>
+      <c r="C330" s="41" t="s">
+        <v>512</v>
+      </c>
+      <c r="D330" s="42" t="s">
+        <v>501</v>
+      </c>
+      <c r="E330" s="39"/>
+      <c r="F330" s="42"/>
+      <c r="G330" s="42"/>
+      <c r="H330" s="42"/>
+      <c r="I330" s="42"/>
+      <c r="J330" s="42"/>
+      <c r="K330" s="42"/>
+    </row>
+    <row r="331" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A331" s="39"/>
+      <c r="B331" s="42"/>
+      <c r="C331" s="41" t="s">
+        <v>513</v>
+      </c>
+      <c r="D331" s="42" t="s">
+        <v>502</v>
+      </c>
+      <c r="E331" s="39"/>
+      <c r="F331" s="42"/>
+      <c r="G331" s="42"/>
+      <c r="H331" s="42"/>
+      <c r="I331" s="42"/>
+      <c r="J331" s="42"/>
+      <c r="K331" s="42"/>
+    </row>
+    <row r="332" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A332" s="39"/>
+      <c r="B332" s="42"/>
+      <c r="C332" s="41" t="s">
+        <v>514</v>
+      </c>
+      <c r="D332" s="42" t="s">
+        <v>515</v>
+      </c>
+      <c r="E332" s="39"/>
+      <c r="F332" s="42"/>
+      <c r="G332" s="42"/>
+      <c r="H332" s="42"/>
+      <c r="I332" s="42"/>
+      <c r="J332" s="42"/>
+      <c r="K332" s="42"/>
+    </row>
+    <row r="333" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A333" s="26"/>
+      <c r="B333" s="25"/>
+      <c r="C333" s="26"/>
+      <c r="D333" s="25"/>
+      <c r="E333" s="26"/>
+      <c r="F333" s="25"/>
+      <c r="G333" s="25"/>
+      <c r="H333" s="25"/>
+      <c r="I333" s="25"/>
+      <c r="J333" s="25"/>
+      <c r="K333" s="25"/>
+    </row>
+    <row r="334" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A334" s="32"/>
+      <c r="B334" s="33" t="s">
         <v>555</v>
       </c>
-      <c r="C328" s="32" t="s">
+      <c r="C334" s="32" t="s">
         <v>556</v>
       </c>
-      <c r="D328" s="38" t="s">
+      <c r="D334" s="38" t="s">
         <v>557</v>
       </c>
-      <c r="E328" s="32"/>
-      <c r="F328" s="33"/>
-      <c r="G328" s="33"/>
-    </row>
-    <row r="329" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A329" s="4"/>
-      <c r="B329" s="5"/>
-      <c r="C329" s="4" t="s">
-        <v>558</v>
-      </c>
-      <c r="D329" s="18" t="s">
-        <v>559</v>
-      </c>
-      <c r="E329" s="4"/>
-      <c r="F329" s="5"/>
-      <c r="G329" s="5"/>
-    </row>
-    <row r="331" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A331" s="4"/>
-      <c r="B331" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="C331" s="4" t="s">
-        <v>560</v>
-      </c>
-      <c r="D331" s="16" t="s">
-        <v>560</v>
-      </c>
-      <c r="E331" s="4"/>
-      <c r="F331" s="5"/>
-      <c r="G331" s="5"/>
-    </row>
-    <row r="332" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A332" s="4"/>
-      <c r="B332" s="5"/>
-      <c r="C332" s="4" t="s">
-        <v>561</v>
-      </c>
-      <c r="D332" s="16" t="s">
-        <v>561</v>
-      </c>
-      <c r="E332" s="4"/>
-      <c r="F332" s="5"/>
-      <c r="G332" s="5"/>
-    </row>
-    <row r="333" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A333" s="4"/>
-      <c r="B333" s="5"/>
-      <c r="C333" s="4" t="s">
-        <v>562</v>
-      </c>
-      <c r="D333" s="16" t="s">
-        <v>562</v>
-      </c>
-      <c r="E333" s="4"/>
-      <c r="F333" s="5"/>
-      <c r="G333" s="5"/>
-    </row>
-    <row r="334" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A334" s="4"/>
-      <c r="B334" s="5"/>
-      <c r="C334" s="4" t="s">
-        <v>563</v>
-      </c>
-      <c r="D334" s="16" t="s">
-        <v>563</v>
-      </c>
-      <c r="E334" s="4"/>
-      <c r="F334" s="5"/>
-      <c r="G334" s="5"/>
+      <c r="E334" s="32"/>
+      <c r="F334" s="33"/>
+      <c r="G334" s="33"/>
     </row>
     <row r="335" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A335" s="4"/>
       <c r="B335" s="5"/>
       <c r="C335" s="4" t="s">
-        <v>564</v>
-      </c>
-      <c r="D335" s="16" t="s">
-        <v>564</v>
+        <v>558</v>
+      </c>
+      <c r="D335" s="18" t="s">
+        <v>559</v>
       </c>
       <c r="E335" s="4"/>
       <c r="F335" s="5"/>
       <c r="G335" s="5"/>
     </row>
-    <row r="336" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A336" s="4"/>
-      <c r="B336" s="5"/>
-      <c r="C336" s="4"/>
-      <c r="D336" s="5"/>
-      <c r="E336" s="4"/>
-      <c r="F336" s="5"/>
-      <c r="G336" s="5"/>
-    </row>
     <row r="337" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A337" s="4"/>
       <c r="B337" s="5" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C337" s="4" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="D337" s="16" t="s">
-        <v>581</v>
+        <v>560</v>
       </c>
       <c r="E337" s="4"/>
-      <c r="F337" s="5" t="s">
-        <v>578</v>
-      </c>
+      <c r="F337" s="5"/>
       <c r="G337" s="5"/>
     </row>
     <row r="338" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A338" s="4"/>
       <c r="B338" s="5"/>
       <c r="C338" s="4" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
       <c r="D338" s="16" t="s">
-        <v>582</v>
+        <v>561</v>
       </c>
       <c r="E338" s="4"/>
-      <c r="F338" s="5" t="s">
-        <v>579</v>
-      </c>
+      <c r="F338" s="5"/>
       <c r="G338" s="5"/>
     </row>
     <row r="339" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A339" s="4"/>
       <c r="B339" s="5"/>
       <c r="C339" s="4" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
       <c r="D339" s="16" t="s">
-        <v>583</v>
+        <v>562</v>
       </c>
       <c r="E339" s="4"/>
-      <c r="F339" s="5" t="s">
-        <v>580</v>
-      </c>
+      <c r="F339" s="5"/>
       <c r="G339" s="5"/>
     </row>
     <row r="340" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A340" s="4"/>
       <c r="B340" s="5"/>
       <c r="C340" s="4" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="D340" s="16" t="s">
-        <v>585</v>
+        <v>563</v>
       </c>
       <c r="E340" s="4"/>
-      <c r="F340" s="5" t="s">
-        <v>584</v>
-      </c>
+      <c r="F340" s="5"/>
       <c r="G340" s="5"/>
     </row>
     <row r="341" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A341" s="4"/>
       <c r="B341" s="5"/>
       <c r="C341" s="4" t="s">
-        <v>571</v>
+        <v>564</v>
       </c>
       <c r="D341" s="16" t="s">
-        <v>571</v>
+        <v>564</v>
       </c>
       <c r="E341" s="4"/>
       <c r="F341" s="5"/>
@@ -7032,69 +6999,409 @@
     <row r="343" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A343" s="4"/>
       <c r="B343" s="5" t="s">
-        <v>572</v>
+        <v>567</v>
       </c>
       <c r="C343" s="4" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="D343" s="16" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="E343" s="4"/>
-      <c r="F343" s="5"/>
+      <c r="F343" s="5" t="s">
+        <v>578</v>
+      </c>
       <c r="G343" s="5"/>
     </row>
     <row r="344" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A344" s="4"/>
       <c r="B344" s="5"/>
       <c r="C344" s="4" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="D344" s="16" t="s">
-        <v>574</v>
+        <v>582</v>
       </c>
       <c r="E344" s="4"/>
-      <c r="F344" s="5"/>
+      <c r="F344" s="5" t="s">
+        <v>579</v>
+      </c>
       <c r="G344" s="5"/>
     </row>
     <row r="345" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A345" s="4"/>
       <c r="B345" s="5"/>
       <c r="C345" s="4" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="D345" s="16" t="s">
-        <v>575</v>
+        <v>583</v>
       </c>
       <c r="E345" s="4"/>
-      <c r="F345" s="5"/>
+      <c r="F345" s="5" t="s">
+        <v>580</v>
+      </c>
       <c r="G345" s="5"/>
     </row>
     <row r="346" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A346" s="4"/>
       <c r="B346" s="5"/>
       <c r="C346" s="4" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="D346" s="16" t="s">
-        <v>576</v>
+        <v>585</v>
       </c>
       <c r="E346" s="4"/>
-      <c r="F346" s="5"/>
+      <c r="F346" s="5" t="s">
+        <v>584</v>
+      </c>
       <c r="G346" s="5"/>
     </row>
     <row r="347" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A347" s="4"/>
       <c r="B347" s="5"/>
       <c r="C347" s="4" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="D347" s="16" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="E347" s="4"/>
       <c r="F347" s="5"/>
       <c r="G347" s="5"/>
+    </row>
+    <row r="348" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A348" s="4"/>
+      <c r="B348" s="5"/>
+      <c r="C348" s="4"/>
+      <c r="D348" s="5"/>
+      <c r="E348" s="4"/>
+      <c r="F348" s="5"/>
+      <c r="G348" s="5"/>
+    </row>
+    <row r="349" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A349" s="4"/>
+      <c r="B349" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="C349" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="D349" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="E349" s="4"/>
+      <c r="F349" s="5"/>
+      <c r="G349" s="5"/>
+    </row>
+    <row r="350" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A350" s="4"/>
+      <c r="B350" s="5"/>
+      <c r="C350" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="D350" s="16" t="s">
+        <v>574</v>
+      </c>
+      <c r="E350" s="4"/>
+      <c r="F350" s="5"/>
+      <c r="G350" s="5"/>
+    </row>
+    <row r="351" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A351" s="4"/>
+      <c r="B351" s="5"/>
+      <c r="C351" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="D351" s="16" t="s">
+        <v>575</v>
+      </c>
+      <c r="E351" s="4"/>
+      <c r="F351" s="5"/>
+      <c r="G351" s="5"/>
+    </row>
+    <row r="352" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A352" s="4"/>
+      <c r="B352" s="5"/>
+      <c r="C352" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="D352" s="16" t="s">
+        <v>576</v>
+      </c>
+      <c r="E352" s="4"/>
+      <c r="F352" s="5"/>
+      <c r="G352" s="5"/>
+    </row>
+    <row r="353" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A353" s="4"/>
+      <c r="B353" s="5"/>
+      <c r="C353" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="D353" s="16" t="s">
+        <v>577</v>
+      </c>
+      <c r="E353" s="4"/>
+      <c r="F353" s="5"/>
+      <c r="G353" s="5"/>
+    </row>
+    <row r="356" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A356" s="43">
+        <v>20</v>
+      </c>
+      <c r="B356" s="44" t="s">
+        <v>701</v>
+      </c>
+      <c r="C356" s="43" t="s">
+        <v>702</v>
+      </c>
+      <c r="D356" s="45" t="s">
+        <v>704</v>
+      </c>
+      <c r="E356" s="43" t="s">
+        <v>706</v>
+      </c>
+      <c r="F356" s="44"/>
+      <c r="G356" s="44"/>
+      <c r="H356" s="44"/>
+      <c r="I356" s="44"/>
+      <c r="J356" s="44"/>
+      <c r="K356" s="44"/>
+    </row>
+    <row r="357" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A357" s="43"/>
+      <c r="B357" s="44"/>
+      <c r="C357" s="43" t="s">
+        <v>703</v>
+      </c>
+      <c r="D357" s="45" t="s">
+        <v>705</v>
+      </c>
+      <c r="E357" s="43" t="s">
+        <v>706</v>
+      </c>
+      <c r="F357" s="44"/>
+      <c r="G357" s="44"/>
+      <c r="H357" s="44"/>
+      <c r="I357" s="44"/>
+      <c r="J357" s="44"/>
+      <c r="K357" s="44"/>
+    </row>
+    <row r="358" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A358" s="43"/>
+      <c r="B358" s="44"/>
+      <c r="C358" s="43" t="s">
+        <v>707</v>
+      </c>
+      <c r="D358" s="44" t="s">
+        <v>708</v>
+      </c>
+      <c r="E358" s="43" t="s">
+        <v>709</v>
+      </c>
+      <c r="F358" s="44"/>
+      <c r="G358" s="44"/>
+      <c r="H358" s="44"/>
+      <c r="I358" s="44"/>
+      <c r="J358" s="44"/>
+      <c r="K358" s="44"/>
+    </row>
+    <row r="359" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A359" s="43"/>
+      <c r="B359" s="44"/>
+      <c r="C359" s="43"/>
+      <c r="D359" s="44"/>
+      <c r="E359" s="43"/>
+      <c r="F359" s="44"/>
+      <c r="G359" s="44"/>
+      <c r="H359" s="44"/>
+      <c r="I359" s="44"/>
+      <c r="J359" s="44"/>
+      <c r="K359" s="44"/>
+    </row>
+    <row r="360" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A360" s="43"/>
+      <c r="B360" s="44"/>
+      <c r="C360" s="43"/>
+      <c r="D360" s="44"/>
+      <c r="E360" s="43"/>
+      <c r="F360" s="44"/>
+      <c r="G360" s="44"/>
+      <c r="H360" s="44"/>
+      <c r="I360" s="44"/>
+      <c r="J360" s="44"/>
+      <c r="K360" s="44"/>
+    </row>
+    <row r="361" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A361" s="43"/>
+      <c r="B361" s="44"/>
+      <c r="C361" s="43"/>
+      <c r="D361" s="44"/>
+      <c r="E361" s="43"/>
+      <c r="F361" s="44"/>
+      <c r="G361" s="44"/>
+      <c r="H361" s="44"/>
+      <c r="I361" s="44"/>
+      <c r="J361" s="44"/>
+      <c r="K361" s="44"/>
+    </row>
+    <row r="362" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A362" s="43"/>
+      <c r="B362" s="44"/>
+      <c r="C362" s="43"/>
+      <c r="D362" s="44"/>
+      <c r="E362" s="43"/>
+      <c r="F362" s="44"/>
+      <c r="G362" s="44"/>
+      <c r="H362" s="44"/>
+      <c r="I362" s="44"/>
+      <c r="J362" s="44"/>
+      <c r="K362" s="44"/>
+    </row>
+    <row r="363" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A363" s="43"/>
+      <c r="B363" s="44"/>
+      <c r="C363" s="43"/>
+      <c r="D363" s="44"/>
+      <c r="E363" s="43"/>
+      <c r="F363" s="44"/>
+      <c r="G363" s="44"/>
+      <c r="H363" s="44"/>
+      <c r="I363" s="44"/>
+      <c r="J363" s="44"/>
+      <c r="K363" s="44"/>
+    </row>
+    <row r="364" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A364" s="43"/>
+      <c r="B364" s="44"/>
+      <c r="C364" s="43"/>
+      <c r="D364" s="44"/>
+      <c r="E364" s="43"/>
+      <c r="F364" s="44"/>
+      <c r="G364" s="44"/>
+      <c r="H364" s="44"/>
+      <c r="I364" s="44"/>
+      <c r="J364" s="44"/>
+      <c r="K364" s="44"/>
+    </row>
+    <row r="365" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A365" s="43"/>
+      <c r="B365" s="44"/>
+      <c r="C365" s="43"/>
+      <c r="D365" s="44"/>
+      <c r="E365" s="43"/>
+      <c r="F365" s="44"/>
+      <c r="G365" s="44"/>
+      <c r="H365" s="44"/>
+      <c r="I365" s="44"/>
+      <c r="J365" s="44"/>
+      <c r="K365" s="44"/>
+    </row>
+    <row r="366" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A366" s="43"/>
+      <c r="B366" s="44"/>
+      <c r="C366" s="43"/>
+      <c r="D366" s="44"/>
+      <c r="E366" s="43"/>
+      <c r="F366" s="44"/>
+      <c r="G366" s="44"/>
+      <c r="H366" s="44"/>
+      <c r="I366" s="44"/>
+      <c r="J366" s="44"/>
+      <c r="K366" s="44"/>
+    </row>
+    <row r="367" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A367" s="43"/>
+      <c r="B367" s="44"/>
+      <c r="C367" s="43"/>
+      <c r="D367" s="44"/>
+      <c r="E367" s="43"/>
+      <c r="F367" s="44"/>
+      <c r="G367" s="44"/>
+      <c r="H367" s="44"/>
+      <c r="I367" s="44"/>
+      <c r="J367" s="44"/>
+      <c r="K367" s="44"/>
+    </row>
+    <row r="368" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A368" s="43"/>
+      <c r="B368" s="44"/>
+      <c r="C368" s="43"/>
+      <c r="D368" s="44"/>
+      <c r="E368" s="43"/>
+      <c r="F368" s="44"/>
+      <c r="G368" s="44"/>
+      <c r="H368" s="44"/>
+      <c r="I368" s="44"/>
+      <c r="J368" s="44"/>
+      <c r="K368" s="44"/>
+    </row>
+    <row r="369" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A369" s="43"/>
+      <c r="B369" s="44"/>
+      <c r="C369" s="43"/>
+      <c r="D369" s="44"/>
+      <c r="E369" s="43"/>
+      <c r="F369" s="44"/>
+      <c r="G369" s="44"/>
+      <c r="H369" s="44"/>
+      <c r="I369" s="44"/>
+      <c r="J369" s="44"/>
+      <c r="K369" s="44"/>
+    </row>
+    <row r="370" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A370" s="43"/>
+      <c r="B370" s="44"/>
+      <c r="C370" s="43"/>
+      <c r="D370" s="44"/>
+      <c r="E370" s="43"/>
+      <c r="F370" s="44"/>
+      <c r="G370" s="44"/>
+      <c r="H370" s="44"/>
+      <c r="I370" s="44"/>
+      <c r="J370" s="44"/>
+      <c r="K370" s="44"/>
+    </row>
+    <row r="371" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A371" s="43"/>
+      <c r="B371" s="44"/>
+      <c r="C371" s="43"/>
+      <c r="D371" s="44"/>
+      <c r="E371" s="43"/>
+      <c r="F371" s="44"/>
+      <c r="G371" s="44"/>
+      <c r="H371" s="44"/>
+      <c r="I371" s="44"/>
+      <c r="J371" s="44"/>
+      <c r="K371" s="44"/>
+    </row>
+    <row r="372" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A372" s="43"/>
+      <c r="B372" s="44"/>
+      <c r="C372" s="43"/>
+      <c r="D372" s="44"/>
+      <c r="E372" s="43"/>
+      <c r="F372" s="44"/>
+      <c r="G372" s="44"/>
+      <c r="H372" s="44"/>
+      <c r="I372" s="44"/>
+      <c r="J372" s="44"/>
+      <c r="K372" s="44"/>
+    </row>
+    <row r="373" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A373" s="43"/>
+      <c r="B373" s="44"/>
+      <c r="C373" s="43"/>
+      <c r="D373" s="44"/>
+      <c r="E373" s="43"/>
+      <c r="F373" s="44"/>
+      <c r="G373" s="44"/>
+      <c r="H373" s="44"/>
+      <c r="I373" s="44"/>
+      <c r="J373" s="44"/>
+      <c r="K373" s="44"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>